<commit_message>
feat(employees): import command for employees.xlsx
</commit_message>
<xml_diff>
--- a/employees.xlsx
+++ b/employees.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GhithOps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B5B21419-3D61-49AF-ABF9-218EB15465B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF8A5765-68A7-4D32-94EB-F9C7590B1F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B72FDE8D-3B47-4238-9363-C8829189ED63}"/>
   </bookViews>
@@ -4227,18 +4227,12 @@
     <t>رضوان عبدالقوي عبدالباقي سيف</t>
   </si>
   <si>
-    <t>موقع سكن الموظف</t>
-  </si>
-  <si>
     <t>نوع الخدمة</t>
   </si>
   <si>
     <t>نوع الدوام</t>
   </si>
   <si>
-    <t>الشركة</t>
-  </si>
-  <si>
     <t>الوظيفة</t>
   </si>
   <si>
@@ -4255,6 +4249,12 @@
   </si>
   <si>
     <t>الحالة</t>
+  </si>
+  <si>
+    <t>موقع السكن</t>
+  </si>
+  <si>
+    <t>الشركة المستفيدة</t>
   </si>
 </sst>
 </file>
@@ -4759,34 +4759,34 @@
   <sheetData>
     <row r="1" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="15" t="s">
+        <v>1405</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>1404</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>1403</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>1402</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>1401</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>1400</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>1399</v>
+      </c>
+      <c r="H1" s="15" t="s">
         <v>1407</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="I1" s="15" t="s">
         <v>1406</v>
       </c>
-      <c r="C1" s="15" t="s">
-        <v>1405</v>
-      </c>
-      <c r="D1" s="15" t="s">
-        <v>1404</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>1403</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>1401</v>
-      </c>
-      <c r="G1" s="15" t="s">
-        <v>1400</v>
-      </c>
-      <c r="H1" s="15" t="s">
-        <v>1399</v>
-      </c>
-      <c r="I1" s="15" t="s">
+      <c r="J1" s="15" t="s">
         <v>1408</v>
-      </c>
-      <c r="J1" s="15" t="s">
-        <v>1402</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="21.75" x14ac:dyDescent="0.2">

</xml_diff>